<commit_message>
changed from protocol to protocol & architecture style for gRPC, REST
</commit_message>
<xml_diff>
--- a/results/ACTUALRESULTS.xlsx
+++ b/results/ACTUALRESULTS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audricho\Documents\ForOfficialDemo\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2657A02F-82E4-4438-ABD5-0070EF04B86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73578C2C-3435-431D-98B3-EF6D6C37A451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BFC95034-0712-4A02-8952-872159A7A178}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="80">
   <si>
     <t>stubGRPCPeoplePeopleInfoServiceStub P-R</t>
   </si>
@@ -371,6 +371,9 @@
   </si>
   <si>
     <t>(Lower Better)</t>
+  </si>
+  <si>
+    <t>Protocol / Architecture Type</t>
   </si>
 </sst>
 </file>
@@ -791,8 +794,8 @@
   <sheetFormatPr defaultColWidth="7.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="7.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="7.77734375" style="1" customWidth="1"/>
-    <col min="4" max="18" width="13.21875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" style="1" customWidth="1"/>
+    <col min="4" max="18" width="13.77734375" style="1" customWidth="1"/>
     <col min="19" max="16384" width="7.77734375" style="1"/>
   </cols>
   <sheetData>
@@ -3523,7 +3526,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>0</v>
       </c>
@@ -3531,7 +3534,7 @@
         <v>212</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>19</v>
+        <v>79</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>16</v>
@@ -3688,7 +3691,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>3</v>
       </c>
@@ -3820,7 +3823,7 @@
         <v>2056.3000000000002</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>2</v>
       </c>
@@ -3891,7 +3894,7 @@
         <v>0.61143801974420064</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>3</v>
       </c>
@@ -9563,7 +9566,7 @@
     <col min="15" max="15" width="16.77734375" customWidth="1"/>
     <col min="16" max="16" width="15.6640625" customWidth="1"/>
     <col min="26" max="26" width="8.88671875" customWidth="1"/>
-    <col min="27" max="27" width="7.77734375" customWidth="1"/>
+    <col min="27" max="27" width="11.33203125" customWidth="1"/>
     <col min="28" max="42" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9964,9 +9967,9 @@
       <c r="AO20" s="1"/>
       <c r="AP20" s="1"/>
     </row>
-    <row r="21" spans="27:42" x14ac:dyDescent="0.3">
+    <row r="21" spans="27:42" ht="72" x14ac:dyDescent="0.3">
       <c r="AA21" s="1" t="s">
-        <v>19</v>
+        <v>79</v>
       </c>
       <c r="AB21" s="1" t="s">
         <v>16</v>

</xml_diff>